<commit_message>
unified plot visualization for nn + predictions 2030 MLP
</commit_message>
<xml_diff>
--- a/results/errors/model_performances.xlsx
+++ b/results/errors/model_performances.xlsx
@@ -463,7 +463,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Cereal yield (kg per hectare)</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -473,23 +473,23 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Random_orig</t>
+          <t>Random_jitter_aug</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>4.2265</v>
+        <v>348.3092</v>
       </c>
       <c r="E2" t="n">
-        <v>3.571</v>
+        <v>269.0354</v>
       </c>
       <c r="F2" t="n">
-        <v>3.76</v>
+        <v>5.34</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Cereal yield (kg per hectare)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -499,23 +499,23 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Random_step_aug</t>
+          <t>Random_orig</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.2432</v>
+        <v>323.3604</v>
       </c>
       <c r="E3" t="n">
-        <v>1.899</v>
+        <v>276.6048</v>
       </c>
       <c r="F3" t="n">
-        <v>1.97</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Cereal yield (kg per hectare)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -525,23 +525,23 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Random_jitter_aug</t>
+          <t>Random_step_aug</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2.6723</v>
+        <v>348.4039</v>
       </c>
       <c r="E4" t="n">
-        <v>2.2791</v>
+        <v>278.7667</v>
       </c>
       <c r="F4" t="n">
-        <v>2.38</v>
+        <v>5.41</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Cereal yield (kg per hectare)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -551,23 +551,23 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>TPE_orig</t>
+          <t>TPE_jitter_aug</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>4.9207</v>
+        <v>352.6013</v>
       </c>
       <c r="E5" t="n">
-        <v>4.5813</v>
+        <v>298.9495</v>
       </c>
       <c r="F5" t="n">
-        <v>4.81</v>
+        <v>5.77</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Cereal yield (kg per hectare)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -577,23 +577,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>TPE_step_aug</t>
+          <t>TPE_orig</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2.8754</v>
+        <v>353.1389</v>
       </c>
       <c r="E6" t="n">
-        <v>2.6153</v>
+        <v>283.6457</v>
       </c>
       <c r="F6" t="n">
-        <v>2.73</v>
+        <v>5.56</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Cereal yield (kg per hectare)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -603,23 +603,23 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>TPE_jitter_aug</t>
+          <t>TPE_step_aug</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3.0573</v>
+        <v>367.5561</v>
       </c>
       <c r="E7" t="n">
-        <v>2.8531</v>
+        <v>279.1253</v>
       </c>
       <c r="F7" t="n">
-        <v>2.98</v>
+        <v>5.48</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Rural population (% of total population)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -629,23 +629,23 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Random_orig</t>
+          <t>Random_jitter_aug</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7.5406</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="E8" t="n">
-        <v>7.295</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>7.66</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Rural population (% of total population)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -655,23 +655,23 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Random_step_aug</t>
+          <t>Random_orig</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3.2975</v>
+        <v>1.4355</v>
       </c>
       <c r="E9" t="n">
-        <v>3.0677</v>
+        <v>1.4137</v>
       </c>
       <c r="F9" t="n">
-        <v>3.21</v>
+        <v>4.96</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Rural population (% of total population)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -681,23 +681,23 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Random_jitter_aug</t>
+          <t>Random_step_aug</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4.9171</v>
+        <v>0.1061</v>
       </c>
       <c r="E10" t="n">
-        <v>4.6952</v>
+        <v>0.1054</v>
       </c>
       <c r="F10" t="n">
-        <v>4.96</v>
+        <v>0.37</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Rural population (% of total population)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -707,23 +707,23 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TPE_orig</t>
+          <t>TPE_jitter_aug</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>4.4922</v>
+        <v>0.5635</v>
       </c>
       <c r="E11" t="n">
-        <v>4.2011</v>
+        <v>0.5556</v>
       </c>
       <c r="F11" t="n">
-        <v>4.42</v>
+        <v>1.95</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Rural population (% of total population)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -733,23 +733,23 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TPE_step_aug</t>
+          <t>TPE_orig</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2.5434</v>
+        <v>1.2361</v>
       </c>
       <c r="E12" t="n">
-        <v>2.3247</v>
+        <v>1.2113</v>
       </c>
       <c r="F12" t="n">
-        <v>2.42</v>
+        <v>4.25</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Crop production index (2014-2016 = 100)</t>
+          <t>Rural population (% of total population)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -759,17 +759,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TPE_jitter_aug</t>
+          <t>TPE_step_aug</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>4.7291</v>
+        <v>0.7779</v>
       </c>
       <c r="E13" t="n">
-        <v>4.3606</v>
+        <v>0.7764</v>
       </c>
       <c r="F13" t="n">
-        <v>4.58</v>
+        <v>2.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
progress in shallow cnn framework
</commit_message>
<xml_diff>
--- a/results/errors/model_performances.xlsx
+++ b/results/errors/model_performances.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,13 +477,13 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.4135</v>
+        <v>0.1839</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4072</v>
+        <v>0.1707</v>
       </c>
       <c r="F2" t="n">
-        <v>24.09</v>
+        <v>9.890000000000001</v>
       </c>
     </row>
     <row r="3">
@@ -503,13 +503,13 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.1975</v>
+        <v>0.2342</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1871</v>
+        <v>0.2278</v>
       </c>
       <c r="F3" t="n">
-        <v>10.72</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="4">
@@ -529,13 +529,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.1212</v>
+        <v>0.1441</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0982</v>
+        <v>0.1265</v>
       </c>
       <c r="F4" t="n">
-        <v>5.65</v>
+        <v>7.35</v>
       </c>
     </row>
     <row r="5">
@@ -555,13 +555,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.4773</v>
+        <v>0.1727</v>
       </c>
       <c r="E5" t="n">
-        <v>0.471</v>
+        <v>0.1528</v>
       </c>
       <c r="F5" t="n">
-        <v>27.85</v>
+        <v>8.710000000000001</v>
       </c>
     </row>
     <row r="6">
@@ -581,13 +581,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.1164</v>
+        <v>0.1792</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0941</v>
+        <v>0.1681</v>
       </c>
       <c r="F6" t="n">
-        <v>5.37</v>
+        <v>9.69</v>
       </c>
     </row>
     <row r="7">
@@ -607,13 +607,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1.8332</v>
+        <v>1.3497</v>
       </c>
       <c r="E7" t="n">
-        <v>1.8257</v>
+        <v>1.3471</v>
       </c>
       <c r="F7" t="n">
-        <v>107.6</v>
+        <v>79.31999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>348.3092</v>
+        <v>345.5138</v>
       </c>
       <c r="E13" t="n">
-        <v>269.0354</v>
+        <v>302.0347</v>
       </c>
       <c r="F13" t="n">
-        <v>5.34</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="14">
@@ -789,13 +789,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>323.3604</v>
+        <v>359.1326</v>
       </c>
       <c r="E14" t="n">
-        <v>276.6048</v>
+        <v>291.2663</v>
       </c>
       <c r="F14" t="n">
-        <v>5.29</v>
+        <v>5.72</v>
       </c>
     </row>
     <row r="15">
@@ -815,13 +815,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>348.4039</v>
+        <v>372.3863</v>
       </c>
       <c r="E15" t="n">
-        <v>278.7667</v>
+        <v>272.9762</v>
       </c>
       <c r="F15" t="n">
-        <v>5.41</v>
+        <v>5.38</v>
       </c>
     </row>
     <row r="16">
@@ -841,13 +841,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>352.6013</v>
+        <v>354.592</v>
       </c>
       <c r="E16" t="n">
-        <v>298.9495</v>
+        <v>289.7007</v>
       </c>
       <c r="F16" t="n">
-        <v>5.77</v>
+        <v>5.63</v>
       </c>
     </row>
     <row r="17">
@@ -867,13 +867,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>353.1389</v>
+        <v>382.7099</v>
       </c>
       <c r="E17" t="n">
-        <v>283.6457</v>
+        <v>295.0389</v>
       </c>
       <c r="F17" t="n">
-        <v>5.56</v>
+        <v>5.86</v>
       </c>
     </row>
     <row r="18">
@@ -893,19 +893,19 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>367.5561</v>
+        <v>364.5954</v>
       </c>
       <c r="E18" t="n">
-        <v>279.1253</v>
+        <v>269.0448</v>
       </c>
       <c r="F18" t="n">
-        <v>5.48</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -919,19 +919,19 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>67.8035</v>
+        <v>0.329</v>
       </c>
       <c r="E19" t="n">
-        <v>64.0655</v>
+        <v>0.2977</v>
       </c>
       <c r="F19" t="n">
-        <v>62.2</v>
+        <v>8.17</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -945,19 +945,19 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>74.4323</v>
+        <v>0.1627</v>
       </c>
       <c r="E20" t="n">
-        <v>71.0329</v>
+        <v>0.132</v>
       </c>
       <c r="F20" t="n">
-        <v>68.45</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -971,19 +971,19 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>73.96420000000001</v>
+        <v>0.1508</v>
       </c>
       <c r="E21" t="n">
-        <v>73.4717</v>
+        <v>0.1211</v>
       </c>
       <c r="F21" t="n">
-        <v>70.26000000000001</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -997,19 +997,19 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>74.90049999999999</v>
+        <v>0.216</v>
       </c>
       <c r="E22" t="n">
-        <v>70.4849</v>
+        <v>0.2139</v>
       </c>
       <c r="F22" t="n">
-        <v>68.73</v>
+        <v>5.82</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1023,19 +1023,19 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>85.0711</v>
+        <v>0.06660000000000001</v>
       </c>
       <c r="E23" t="n">
-        <v>77.18819999999999</v>
+        <v>0.0571</v>
       </c>
       <c r="F23" t="n">
-        <v>77.18000000000001</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (% of fertilizer production)</t>
+          <t>Employment in agriculture (% of total employment)</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1049,19 +1049,19 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>67.0583</v>
+        <v>0.1386</v>
       </c>
       <c r="E24" t="n">
-        <v>61.5235</v>
+        <v>0.1057</v>
       </c>
       <c r="F24" t="n">
-        <v>59.51</v>
+        <v>2.93</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1075,19 +1075,19 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.07539999999999999</v>
+        <v>67.8035</v>
       </c>
       <c r="E25" t="n">
-        <v>0.07190000000000001</v>
+        <v>64.0655</v>
       </c>
       <c r="F25" t="n">
-        <v>0.25</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1101,19 +1101,19 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1.4355</v>
+        <v>74.4323</v>
       </c>
       <c r="E26" t="n">
-        <v>1.4137</v>
+        <v>71.0329</v>
       </c>
       <c r="F26" t="n">
-        <v>4.96</v>
+        <v>68.45</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1127,19 +1127,19 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.1061</v>
+        <v>73.96420000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1054</v>
+        <v>73.4717</v>
       </c>
       <c r="F27" t="n">
-        <v>0.37</v>
+        <v>70.26000000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1153,19 +1153,19 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.5635</v>
+        <v>74.90049999999999</v>
       </c>
       <c r="E28" t="n">
-        <v>0.5556</v>
+        <v>70.4849</v>
       </c>
       <c r="F28" t="n">
-        <v>1.95</v>
+        <v>68.73</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1179,38 +1179,194 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1.2361</v>
+        <v>85.0711</v>
       </c>
       <c r="E29" t="n">
-        <v>1.2113</v>
+        <v>77.18819999999999</v>
       </c>
       <c r="F29" t="n">
-        <v>4.25</v>
+        <v>77.18000000000001</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>TPE_step_aug</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>67.0583</v>
+      </c>
+      <c r="E30" t="n">
+        <v>61.5235</v>
+      </c>
+      <c r="F30" t="n">
+        <v>59.51</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Rural population (% of total population)</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>MLP</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Random_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0.07190000000000001</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Random_orig</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1.4355</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1.4137</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4.96</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Random_step_aug</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0.1061</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0.1054</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>TPE_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0.5635</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0.5556</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>TPE_orig</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>1.2361</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1.2113</v>
+      </c>
+      <c r="F35" t="n">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>TPE_step_aug</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D36" t="n">
         <v>0.7779</v>
       </c>
-      <c r="E30" t="n">
+      <c r="E36" t="n">
         <v>0.7764</v>
       </c>
-      <c r="F30" t="n">
+      <c r="F36" t="n">
         <v>2.72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
different implementation of 2030 forecasting in MLP and tried implementation in CNN
</commit_message>
<xml_diff>
--- a/results/errors/model_performances.xlsx
+++ b/results/errors/model_performances.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -919,13 +919,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.329</v>
+        <v>0.1393</v>
       </c>
       <c r="E19" t="n">
-        <v>0.2977</v>
+        <v>0.1111</v>
       </c>
       <c r="F19" t="n">
-        <v>8.17</v>
+        <v>3.07</v>
       </c>
     </row>
     <row r="20">
@@ -997,13 +997,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.216</v>
+        <v>0.2929</v>
       </c>
       <c r="E22" t="n">
-        <v>0.2139</v>
+        <v>0.2719</v>
       </c>
       <c r="F22" t="n">
-        <v>5.82</v>
+        <v>7.45</v>
       </c>
     </row>
     <row r="23">
@@ -1023,13 +1023,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.1494</v>
       </c>
       <c r="E23" t="n">
-        <v>0.0571</v>
+        <v>0.1293</v>
       </c>
       <c r="F23" t="n">
-        <v>1.57</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="24">
@@ -1049,13 +1049,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.1386</v>
+        <v>0.1683</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1057</v>
+        <v>0.1475</v>
       </c>
       <c r="F24" t="n">
-        <v>2.93</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="25">
@@ -1217,7 +1217,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.07539999999999999</v>
+        <v>8.059799999999999</v>
       </c>
       <c r="E31" t="n">
-        <v>0.07190000000000001</v>
+        <v>5.3619</v>
       </c>
       <c r="F31" t="n">
-        <v>0.25</v>
+        <v>4.65</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1257,19 +1257,19 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.4355</v>
+        <v>7.6108</v>
       </c>
       <c r="E32" t="n">
-        <v>1.4137</v>
+        <v>5.8645</v>
       </c>
       <c r="F32" t="n">
-        <v>4.96</v>
+        <v>5.07</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1283,19 +1283,19 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.1061</v>
+        <v>6.3702</v>
       </c>
       <c r="E33" t="n">
-        <v>0.1054</v>
+        <v>5.866</v>
       </c>
       <c r="F33" t="n">
-        <v>0.37</v>
+        <v>4.84</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1309,19 +1309,19 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.5635</v>
+        <v>6.8937</v>
       </c>
       <c r="E34" t="n">
-        <v>0.5556</v>
+        <v>6.7313</v>
       </c>
       <c r="F34" t="n">
-        <v>1.95</v>
+        <v>5.51</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1335,38 +1335,194 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1.2361</v>
+        <v>7.342</v>
       </c>
       <c r="E35" t="n">
-        <v>1.2113</v>
+        <v>6.9938</v>
       </c>
       <c r="F35" t="n">
-        <v>4.25</v>
+        <v>5.71</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>TPE_step_aug</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>9.274900000000001</v>
+      </c>
+      <c r="E36" t="n">
+        <v>6.7354</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5.89</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>Rural population (% of total population)</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>MLP</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Random_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0.07190000000000001</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Random_orig</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>1.4355</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1.4137</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4.96</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Random_step_aug</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0.1061</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0.1054</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TPE_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0.5635</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0.5556</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TPE_orig</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>1.2361</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1.2113</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
         <is>
           <t>TPE_step_aug</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D42" t="n">
         <v>0.7779</v>
       </c>
-      <c r="E36" t="n">
+      <c r="E42" t="n">
         <v>0.7764</v>
       </c>
-      <c r="F36" t="n">
+      <c r="F42" t="n">
         <v>2.72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
started hyperparameter tuning cnn
</commit_message>
<xml_diff>
--- a/results/errors/model_performances.xlsx
+++ b/results/errors/model_performances.xlsx
@@ -1231,13 +1231,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>8.059799999999999</v>
+        <v>6.3138</v>
       </c>
       <c r="E31" t="n">
-        <v>5.3619</v>
+        <v>5.3866</v>
       </c>
       <c r="F31" t="n">
-        <v>4.65</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="32">
@@ -1257,13 +1257,13 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>7.6108</v>
+        <v>10.9859</v>
       </c>
       <c r="E32" t="n">
-        <v>5.8645</v>
+        <v>8.9224</v>
       </c>
       <c r="F32" t="n">
-        <v>5.07</v>
+        <v>7.07</v>
       </c>
     </row>
     <row r="33">
@@ -1283,13 +1283,13 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>6.3702</v>
+        <v>7.2036</v>
       </c>
       <c r="E33" t="n">
-        <v>5.866</v>
+        <v>4.7265</v>
       </c>
       <c r="F33" t="n">
-        <v>4.84</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="34">
@@ -1309,13 +1309,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6.8937</v>
+        <v>10.6843</v>
       </c>
       <c r="E34" t="n">
-        <v>6.7313</v>
+        <v>8.680099999999999</v>
       </c>
       <c r="F34" t="n">
-        <v>5.51</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="35">
@@ -1335,13 +1335,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7.342</v>
+        <v>18.2856</v>
       </c>
       <c r="E35" t="n">
-        <v>6.9938</v>
+        <v>16.4707</v>
       </c>
       <c r="F35" t="n">
-        <v>5.71</v>
+        <v>13.25</v>
       </c>
     </row>
     <row r="36">
@@ -1361,13 +1361,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>9.274900000000001</v>
+        <v>7.0368</v>
       </c>
       <c r="E36" t="n">
-        <v>6.7354</v>
+        <v>5.8935</v>
       </c>
       <c r="F36" t="n">
-        <v>5.89</v>
+        <v>5.05</v>
       </c>
     </row>
     <row r="37">

</xml_diff>

<commit_message>
Finished 2030 predictions for cnn
</commit_message>
<xml_diff>
--- a/results/errors/model_performances.xlsx
+++ b/results/errors/model_performances.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1066,7 +1066,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1075,13 +1075,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>67.8035</v>
+        <v>47.6128</v>
       </c>
       <c r="E25" t="n">
-        <v>64.0655</v>
+        <v>41.326</v>
       </c>
       <c r="F25" t="n">
-        <v>62.2</v>
+        <v>41.91</v>
       </c>
     </row>
     <row r="26">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1101,13 +1101,13 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>74.4323</v>
+        <v>56.2289</v>
       </c>
       <c r="E26" t="n">
-        <v>71.0329</v>
+        <v>49.2201</v>
       </c>
       <c r="F26" t="n">
-        <v>68.45</v>
+        <v>52.03</v>
       </c>
     </row>
     <row r="27">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1127,13 +1127,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>73.96420000000001</v>
+        <v>71.1495</v>
       </c>
       <c r="E27" t="n">
-        <v>73.4717</v>
+        <v>66.4533</v>
       </c>
       <c r="F27" t="n">
-        <v>70.26000000000001</v>
+        <v>69.01000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1144,7 +1144,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1153,13 +1153,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>74.90049999999999</v>
+        <v>60.8123</v>
       </c>
       <c r="E28" t="n">
-        <v>70.4849</v>
+        <v>57.2434</v>
       </c>
       <c r="F28" t="n">
-        <v>68.73</v>
+        <v>56.17</v>
       </c>
     </row>
     <row r="29">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1179,13 +1179,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>85.0711</v>
+        <v>48.8015</v>
       </c>
       <c r="E29" t="n">
-        <v>77.18819999999999</v>
+        <v>43.9661</v>
       </c>
       <c r="F29" t="n">
-        <v>77.18000000000001</v>
+        <v>44.53</v>
       </c>
     </row>
     <row r="30">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MLP</t>
+          <t>CNN</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1205,19 +1205,19 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>67.0583</v>
+        <v>64.1542</v>
       </c>
       <c r="E30" t="n">
-        <v>61.5235</v>
+        <v>58.7422</v>
       </c>
       <c r="F30" t="n">
-        <v>59.51</v>
+        <v>58.45</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1231,19 +1231,19 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>6.3138</v>
+        <v>67.8035</v>
       </c>
       <c r="E31" t="n">
-        <v>5.3866</v>
+        <v>64.0655</v>
       </c>
       <c r="F31" t="n">
-        <v>4.41</v>
+        <v>62.2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1257,19 +1257,19 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>10.9859</v>
+        <v>74.4323</v>
       </c>
       <c r="E32" t="n">
-        <v>8.9224</v>
+        <v>71.0329</v>
       </c>
       <c r="F32" t="n">
-        <v>7.07</v>
+        <v>68.45</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1283,19 +1283,19 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7.2036</v>
+        <v>73.96420000000001</v>
       </c>
       <c r="E33" t="n">
-        <v>4.7265</v>
+        <v>73.4717</v>
       </c>
       <c r="F33" t="n">
-        <v>4.09</v>
+        <v>70.26000000000001</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1309,19 +1309,19 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>10.6843</v>
+        <v>74.90049999999999</v>
       </c>
       <c r="E34" t="n">
-        <v>8.680099999999999</v>
+        <v>70.4849</v>
       </c>
       <c r="F34" t="n">
-        <v>6.88</v>
+        <v>68.73</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1335,19 +1335,19 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>18.2856</v>
+        <v>85.0711</v>
       </c>
       <c r="E35" t="n">
-        <v>16.4707</v>
+        <v>77.18819999999999</v>
       </c>
       <c r="F35" t="n">
-        <v>13.25</v>
+        <v>77.18000000000001</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+          <t>Fertilizer consumption (% of fertilizer production)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1361,19 +1361,19 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>7.0368</v>
+        <v>67.0583</v>
       </c>
       <c r="E36" t="n">
-        <v>5.8935</v>
+        <v>61.5235</v>
       </c>
       <c r="F36" t="n">
-        <v>5.05</v>
+        <v>59.51</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1387,19 +1387,19 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.07539999999999999</v>
+        <v>6.3138</v>
       </c>
       <c r="E37" t="n">
-        <v>0.07190000000000001</v>
+        <v>5.3866</v>
       </c>
       <c r="F37" t="n">
-        <v>0.25</v>
+        <v>4.41</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1413,19 +1413,19 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.4355</v>
+        <v>10.9859</v>
       </c>
       <c r="E38" t="n">
-        <v>1.4137</v>
+        <v>8.9224</v>
       </c>
       <c r="F38" t="n">
-        <v>4.96</v>
+        <v>7.07</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1439,19 +1439,19 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.1061</v>
+        <v>7.2036</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1054</v>
+        <v>4.7265</v>
       </c>
       <c r="F39" t="n">
-        <v>0.37</v>
+        <v>4.09</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1465,19 +1465,19 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.5635</v>
+        <v>10.6843</v>
       </c>
       <c r="E40" t="n">
-        <v>0.5556</v>
+        <v>8.680099999999999</v>
       </c>
       <c r="F40" t="n">
-        <v>1.95</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rural population (% of total population)</t>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1491,38 +1491,350 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>1.2361</v>
+        <v>18.2856</v>
       </c>
       <c r="E41" t="n">
-        <v>1.2113</v>
+        <v>16.4707</v>
       </c>
       <c r="F41" t="n">
-        <v>4.25</v>
+        <v>13.25</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>Fertilizer consumption (kilograms per hectare of arable land)</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TPE_step_aug</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>7.0368</v>
+      </c>
+      <c r="E42" t="n">
+        <v>5.8935</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5.05</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Random_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>3.7365</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.9597</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Random_orig</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>3.204</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.8476</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2.69</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Random_step_aug</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>4.0386</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3.6203</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3.41</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>TPE_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>3.4649</v>
+      </c>
+      <c r="E46" t="n">
+        <v>2.9408</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2.77</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>TPE_orig</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>3.0275</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.8254</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.68</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Livestock production index (2014-2016 = 100)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>CNN</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>TPE_step_aug</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>3.4904</v>
+      </c>
+      <c r="E48" t="n">
+        <v>3.0109</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2.84</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>Rural population (% of total population)</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>MLP</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Random_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>0.07539999999999999</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0.07190000000000001</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Random_orig</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>1.4355</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1.4137</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4.96</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Random_step_aug</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>0.1061</v>
+      </c>
+      <c r="E51" t="n">
+        <v>0.1054</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.37</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>TPE_jitter_aug</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>0.5635</v>
+      </c>
+      <c r="E52" t="n">
+        <v>0.5556</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>TPE_orig</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>1.2361</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1.2113</v>
+      </c>
+      <c r="F53" t="n">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Rural population (% of total population)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
         <is>
           <t>TPE_step_aug</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D54" t="n">
         <v>0.7779</v>
       </c>
-      <c r="E42" t="n">
+      <c r="E54" t="n">
         <v>0.7764</v>
       </c>
-      <c r="F42" t="n">
+      <c r="F54" t="n">
         <v>2.72</v>
       </c>
     </row>

</xml_diff>